<commit_message>
Daily EOD data and reports for 2026-08-27
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260827.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260827.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.93</v>
+        <v>1.925</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.055</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-2.53%</t>
+          <t>-2.78%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>295639.33</v>
+        <v>294873.42</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-7659.05</v>
+        <v>-8424.950000000001</v>
       </c>
     </row>
     <row r="5">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>66.8</v>
+        <v>66.7</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-1.04%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>9000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>601200</v>
+        <v>600300</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-5400</v>
+        <v>-6300</v>
       </c>
     </row>
     <row r="8">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>132.27</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-132.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>155.32</v>
+        <v>155.86</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.14</v>
+        <v>0.4</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>0.26%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>173.58</v>
+        <v>172.91</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.14</v>
+        <v>0.47</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.66%</t>
+          <t>0.27%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>694320</v>
+        <v>691640</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4560</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0</v>
+        <v>0.285</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.285</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>5700</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-5700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>33.88</v>
+        <v>33.94</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.15%</t>
+          <t>0.33%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.88</v>
+        <v>32.12</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.04</v>
+        <v>0.2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41061.44</v>
+        <v>41370.56</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-51.52</v>
+        <v>257.6</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1808800.77</v>
+        <v>1810596.26</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-82944.02</v>
+        <v>-81148.53999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>